<commit_message>
update: general models update
</commit_message>
<xml_diff>
--- a/Models/CDGP.xlsx
+++ b/Models/CDGP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/36a87f973740ffce/Documents/Personal/Finance/Models/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1030" documentId="8_{AB677FD1-DACE-674B-8687-43CC81DC24D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{83DF83A7-05AE-8D48-B6A8-E43FB98E4561}"/>
+  <xr:revisionPtr revIDLastSave="1039" documentId="8_{AB677FD1-DACE-674B-8687-43CC81DC24D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B27D25B-B159-CB46-9362-EC0AD4176992}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17860" activeTab="1" xr2:uid="{D13D7BE5-6829-5F46-8F18-3C3B077CFA17}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="199">
   <si>
     <t xml:space="preserve">Price </t>
   </si>
@@ -477,9 +477,6 @@
     <t>CFS</t>
   </si>
   <si>
-    <t>Working capital changes</t>
-  </si>
-  <si>
     <t>CapEx</t>
   </si>
   <si>
@@ -634,6 +631,12 @@
   </si>
   <si>
     <t xml:space="preserve">* low WACC &amp; the D/E = industry average </t>
+  </si>
+  <si>
+    <t>ΔNWC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CFF </t>
   </si>
 </sst>
 </file>
@@ -813,15 +816,12 @@
     <xf numFmtId="10" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -840,12 +840,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1203,7 +1206,7 @@
     </row>
     <row r="3" spans="2:13">
       <c r="B3" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="J3" s="5"/>
     </row>
@@ -1211,15 +1214,15 @@
       <c r="B4" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="J4" s="29" t="s">
-        <v>166</v>
-      </c>
-      <c r="K4" s="30"/>
-      <c r="L4" s="31"/>
+      <c r="J4" s="39" t="s">
+        <v>165</v>
+      </c>
+      <c r="K4" s="40"/>
+      <c r="L4" s="41"/>
     </row>
     <row r="5" spans="2:13">
       <c r="B5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="J5" t="s">
         <v>0</v>
@@ -1360,12 +1363,12 @@
       </c>
     </row>
     <row r="18" spans="2:13">
-      <c r="B18" s="29" t="s">
+      <c r="B18" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="30"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="31"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="41"/>
       <c r="J18" t="s">
         <v>7</v>
       </c>
@@ -1389,7 +1392,7 @@
         <v>24</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K20" s="7">
         <f>Model!F44</f>
@@ -1439,7 +1442,7 @@
         <v>-3.7169406719085057E-2</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="K22" s="7">
         <f>K20-K21</f>
@@ -1748,12 +1751,12 @@
       </c>
     </row>
     <row r="40" spans="2:12">
-      <c r="B40" s="29" t="s">
+      <c r="B40" s="39" t="s">
         <v>53</v>
       </c>
-      <c r="C40" s="30"/>
-      <c r="D40" s="30"/>
-      <c r="E40" s="31"/>
+      <c r="C40" s="40"/>
+      <c r="D40" s="40"/>
+      <c r="E40" s="41"/>
     </row>
     <row r="41" spans="2:12">
       <c r="B41" s="6" t="s">
@@ -1927,13 +1930,13 @@
       </c>
     </row>
     <row r="3" spans="1:6" customFormat="1">
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="33" t="s">
         <v>87</v>
       </c>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="34"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="35"/>
     </row>
     <row r="4" spans="1:6" s="7" customFormat="1">
       <c r="A4" s="6"/>
@@ -2240,7 +2243,7 @@
     </row>
     <row r="20" spans="1:7">
       <c r="B20" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C20" s="9">
         <f t="shared" ref="C20:E20" si="1">C19/C18</f>
@@ -2448,13 +2451,13 @@
     </row>
     <row r="36" spans="1:6" s="7" customFormat="1">
       <c r="A36" s="6"/>
-      <c r="B36" s="35" t="s">
+      <c r="B36" s="36" t="s">
         <v>86</v>
       </c>
-      <c r="C36" s="36"/>
-      <c r="D36" s="36"/>
-      <c r="E36" s="36"/>
-      <c r="F36" s="37"/>
+      <c r="C36" s="37"/>
+      <c r="D36" s="37"/>
+      <c r="E36" s="37"/>
+      <c r="F36" s="38"/>
     </row>
     <row r="37" spans="1:6">
       <c r="B37" t="s">
@@ -2983,17 +2986,17 @@
       </c>
     </row>
     <row r="75" spans="1:6">
-      <c r="B75" s="32" t="s">
+      <c r="B75" s="33" t="s">
         <v>144</v>
       </c>
-      <c r="C75" s="33"/>
-      <c r="D75" s="33"/>
-      <c r="E75" s="33"/>
-      <c r="F75" s="34"/>
+      <c r="C75" s="34"/>
+      <c r="D75" s="34"/>
+      <c r="E75" s="34"/>
+      <c r="F75" s="35"/>
     </row>
     <row r="76" spans="1:6">
       <c r="B76" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C76" s="18">
         <v>1078</v>
@@ -3010,7 +3013,7 @@
     </row>
     <row r="77" spans="1:6">
       <c r="B77" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C77" s="8">
         <v>595</v>
@@ -3027,7 +3030,7 @@
     </row>
     <row r="78" spans="1:6">
       <c r="B78" s="8" t="s">
-        <v>145</v>
+        <v>197</v>
       </c>
       <c r="C78" s="8">
         <v>-234</v>
@@ -3045,7 +3048,7 @@
     <row r="79" spans="1:6" s="7" customFormat="1">
       <c r="A79" s="6"/>
       <c r="B79" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C79" s="7">
         <v>1439</v>
@@ -3063,7 +3066,7 @@
     <row r="80" spans="1:6" s="7" customFormat="1">
       <c r="A80" s="6"/>
       <c r="B80" s="6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C80" s="7">
         <v>-1104</v>
@@ -3081,7 +3084,7 @@
     <row r="81" spans="1:6" s="7" customFormat="1">
       <c r="A81" s="6"/>
       <c r="B81" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C81" s="6">
         <v>335</v>
@@ -3098,7 +3101,7 @@
     </row>
     <row r="82" spans="1:6">
       <c r="B82" s="8" t="s">
-        <v>150</v>
+        <v>198</v>
       </c>
       <c r="C82" s="18">
         <v>4022</v>
@@ -3115,7 +3118,7 @@
     </row>
     <row r="83" spans="1:6">
       <c r="B83" s="8" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C83" s="18">
         <v>4355</v>
@@ -3132,7 +3135,7 @@
     </row>
     <row r="85" spans="1:6">
       <c r="B85" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D85" s="9">
         <f>C79/D79-1</f>
@@ -3149,7 +3152,7 @@
     </row>
     <row r="86" spans="1:6">
       <c r="B86" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D86" s="9">
         <f>C81/D81-1</f>
@@ -3166,32 +3169,32 @@
     </row>
     <row r="88" spans="1:6">
       <c r="B88" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="89" spans="1:6">
       <c r="B89" s="23" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="90" spans="1:6">
       <c r="B90" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="91" spans="1:6">
       <c r="B91" s="22" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="92" spans="1:6">
       <c r="B92" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="93" spans="1:6">
       <c r="B93" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -3225,75 +3228,75 @@
     </row>
     <row r="2" spans="1:8">
       <c r="B2" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C2" s="24">
         <f>((Main!K7/(Main!K8+Main!K7))*C4)+((Main!K8/(Main!K8+Main!K7))*C10*(1-C13))</f>
         <v>6.885039299464453E-2</v>
       </c>
-      <c r="H2" s="38" t="s">
-        <v>177</v>
+      <c r="H2" s="29" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="C3" s="25"/>
       <c r="H3" s="8" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="B4" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C4" s="24">
         <f>C5+C6*(C8)</f>
         <v>8.7574999999999986E-2</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="B5" s="8" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C5" s="26">
         <v>4.5499999999999999E-2</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="H5" s="8"/>
     </row>
     <row r="6" spans="1:8">
       <c r="B6" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C6" s="25">
         <v>0.99</v>
       </c>
-      <c r="D6" s="39"/>
+      <c r="D6" s="30"/>
       <c r="H6" s="18" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="B7" s="8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C7" s="26">
         <v>8.7999999999999995E-2</v>
       </c>
       <c r="D7" s="16" t="s">
+        <v>170</v>
+      </c>
+      <c r="H7" s="8" t="s">
         <v>171</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="B8" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C8" s="26">
         <f>C7-C5</f>
@@ -3308,19 +3311,19 @@
     </row>
     <row r="10" spans="1:8">
       <c r="B10" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C10" s="24">
         <f>(C11/C12)*(1-C13)</f>
         <v>1.7264378871663585E-2</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="B11" s="27" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C11" s="27">
         <f>Model!F16</f>
@@ -3333,7 +3336,7 @@
     </row>
     <row r="12" spans="1:8">
       <c r="B12" s="27" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C12" s="27">
         <f>Main!K8</f>
@@ -3343,12 +3346,12 @@
         <v>6</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="B13" s="25" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C13" s="28">
         <f>Model!E20</f>
@@ -3358,47 +3361,47 @@
         <v>56</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="H14" s="8" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="15" spans="1:8">
-      <c r="B15" s="40" t="s">
-        <v>175</v>
-      </c>
-      <c r="C15" s="41">
+      <c r="B15" s="31" t="s">
+        <v>174</v>
+      </c>
+      <c r="C15" s="32">
         <f>Main!K21/Main!K22</f>
         <v>0.78752802121917787</v>
       </c>
-      <c r="D15" s="40"/>
+      <c r="D15" s="31"/>
       <c r="H15" s="8" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="B16" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C16" s="2">
         <v>0.78339999999999999</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="17" spans="2:11">
       <c r="C17" s="25"/>
       <c r="H17" s="8" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="18" spans="2:11">
       <c r="B18" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="19" spans="2:11">
@@ -3566,7 +3569,7 @@
         <v>129</v>
       </c>
       <c r="C14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -3574,10 +3577,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C15" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -3585,10 +3588,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C16" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -3596,10 +3599,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
+        <v>152</v>
+      </c>
+      <c r="C17" t="s">
         <v>153</v>
-      </c>
-      <c r="C17" t="s">
-        <v>154</v>
       </c>
     </row>
   </sheetData>

</xml_diff>